<commit_message>
SAM & SOM equations updates with linked sheet
</commit_message>
<xml_diff>
--- a/02_Market_Research/TAM_SAM_SOM_Model.xlsx
+++ b/02_Market_Research/TAM_SAM_SOM_Model.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sidha\Downloads\BA-PgBee-expansion-analytics\02_Market_Research\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85918B9E-D32B-480A-93D5-68801E3CAC4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E53F87D3-159C-427B-A107-85B4C1BCC945}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{0651041D-86AB-47F8-B505-8ABFF177DCCF}"/>
   </bookViews>
@@ -624,8 +624,8 @@
         <v>25</v>
       </c>
       <c r="B8" s="3">
-        <f>B6*B4</f>
-        <v>4995</v>
+        <f>B7*B4</f>
+        <v>159790050</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="42" customHeight="1">
@@ -1102,7 +1102,7 @@
       </c>
       <c r="C3" s="2">
         <f>Market_Summary!B8</f>
-        <v>4995</v>
+        <v>159790050</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="67.8" customHeight="1">

</xml_diff>